<commit_message>
Sprint 4 Administration & Policies
feat: add leave type management REST API
feat: add leave policies UI for HR
feat: implement yearly leave balance generation service
feat: add DB trigger and MySQL event for leave balances
feat: add user administration REST API and service
feat: add HR user administration UI
chore: align JPA entities, DTOs and repositories with DB schema
chore: make repositories transactional to fix JPA errors
docs: update README for Sprint 4 administration and policies
</commit_message>
<xml_diff>
--- a/Modeling/User Stories.xlsx
+++ b/Modeling/User Stories.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\leave-management-system\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\leave-management-system\Modeling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3AF4BBC-A6CA-40C0-BD2B-9E6301821327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC8355FD-6E44-419F-BECE-866374D8D3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{33A6ED59-84CF-4D4E-A9BF-49543882D1FF}"/>
   </bookViews>
@@ -705,9 +705,57 @@
   </cellStyleXfs>
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -726,68 +774,20 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1117,726 +1117,779 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:17" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="O2" s="2" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="O2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="4"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="20"/>
     </row>
     <row r="3" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="28" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="O3" s="5" t="s">
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="O3" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
     </row>
     <row r="4" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="28" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="O4" s="6" t="s">
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="O4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
     </row>
     <row r="5" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="28" t="s">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="O5" s="7" t="s">
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="O5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="28" t="s">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
-      <c r="K6" s="28"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="21"/>
-      <c r="D7" s="28" t="s">
+      <c r="C7" s="4"/>
+      <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="28"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="28" t="s">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="28"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="28" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="28" t="s">
+      <c r="C10" s="5"/>
+      <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="28" t="s">
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
-      <c r="K11" s="28"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="28" t="s">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="J14" s="1" t="s">
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="J14" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="10" t="s">
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="J15" s="27" t="s">
+      <c r="J15" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K15" s="27"/>
-      <c r="L15" s="26" t="s">
+      <c r="K15" s="16"/>
+      <c r="L15" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="M15" s="26"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="26"/>
-      <c r="P15" s="26"/>
+      <c r="M15" s="24"/>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="24"/>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="8" t="s">
+      <c r="C16" s="14"/>
+      <c r="D16" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="10"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="26" t="s">
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="17"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="M16" s="26"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="26"/>
-      <c r="P16" s="26"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="8" t="s">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="10"/>
-      <c r="J17" s="27" t="s">
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="17"/>
+      <c r="J17" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K17" s="27"/>
-      <c r="L17" s="22" t="s">
+      <c r="K17" s="16"/>
+      <c r="L17" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="22"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="8" t="s">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="10"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="22" t="s">
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="17"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
-      <c r="P18" s="22"/>
+      <c r="M18" s="25"/>
+      <c r="N18" s="25"/>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="10"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
-      <c r="L19" s="22" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="17"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="22"/>
-      <c r="P19" s="22"/>
+      <c r="M19" s="25"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="10"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="22" t="s">
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="17"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="22"/>
-      <c r="P20" s="22"/>
+      <c r="M20" s="25"/>
+      <c r="N20" s="25"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="13" t="s">
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="J21" s="27" t="s">
+      <c r="J21" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="K21" s="27"/>
-      <c r="L21" s="25" t="s">
+      <c r="K21" s="16"/>
+      <c r="L21" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="M21" s="25"/>
-      <c r="N21" s="25"/>
-      <c r="O21" s="25"/>
-      <c r="P21" s="25"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="26"/>
+      <c r="P21" s="26"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="8" t="s">
+      <c r="C22" s="14"/>
+      <c r="D22" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="13"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="25" t="s">
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="15"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="M22" s="25"/>
-      <c r="N22" s="25"/>
-      <c r="O22" s="25"/>
-      <c r="P22" s="25"/>
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="26"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="8" t="s">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="13"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="25" t="s">
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="15"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="M23" s="25"/>
-      <c r="N23" s="25"/>
-      <c r="O23" s="25"/>
-      <c r="P23" s="25"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="26"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="8" t="s">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="13"/>
-      <c r="J24" s="27" t="s">
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="15"/>
+      <c r="J24" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="K24" s="27"/>
-      <c r="L24" s="24" t="s">
+      <c r="K24" s="16"/>
+      <c r="L24" s="28" t="s">
         <v>67</v>
       </c>
-      <c r="M24" s="24"/>
-      <c r="N24" s="24"/>
-      <c r="O24" s="24"/>
-      <c r="P24" s="24"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
+      <c r="O24" s="28"/>
+      <c r="P24" s="28"/>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="13"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="24" t="s">
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="15"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="28" t="s">
         <v>68</v>
       </c>
-      <c r="M25" s="24"/>
-      <c r="N25" s="24"/>
-      <c r="O25" s="24"/>
-      <c r="P25" s="24"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28"/>
+      <c r="O25" s="28"/>
+      <c r="P25" s="28"/>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="13"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="24" t="s">
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="15"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="M26" s="24"/>
-      <c r="N26" s="24"/>
-      <c r="O26" s="24"/>
-      <c r="P26" s="24"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
+      <c r="O26" s="28"/>
+      <c r="P26" s="28"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="15" t="s">
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="J27" s="27" t="s">
+      <c r="J27" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="K27" s="27"/>
-      <c r="L27" s="8" t="s">
+      <c r="K27" s="16"/>
+      <c r="L27" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="8"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
+      <c r="O27" s="9"/>
+      <c r="P27" s="9"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="14"/>
-      <c r="D28" s="8" t="s">
+      <c r="C28" s="7"/>
+      <c r="D28" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="15"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="8" t="s">
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="11"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="M28" s="8"/>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="9"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="8" t="s">
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="15"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="8" t="s">
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="11"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="M29" s="8"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
+      <c r="O29" s="9"/>
+      <c r="P29" s="9"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="8" t="s">
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="15"/>
-      <c r="J30" s="27" t="s">
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="11"/>
+      <c r="J30" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="K30" s="27"/>
-      <c r="L30" s="23" t="s">
+      <c r="K30" s="16"/>
+      <c r="L30" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="M30" s="23"/>
-      <c r="N30" s="23"/>
-      <c r="O30" s="23"/>
-      <c r="P30" s="23"/>
+      <c r="M30" s="27"/>
+      <c r="N30" s="27"/>
+      <c r="O30" s="27"/>
+      <c r="P30" s="27"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="15"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="23" t="s">
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="11"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="M31" s="23"/>
-      <c r="N31" s="23"/>
-      <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="M31" s="27"/>
+      <c r="N31" s="27"/>
+      <c r="O31" s="27"/>
+      <c r="P31" s="27"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="9"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="9"/>
-      <c r="H32" s="15"/>
-      <c r="J32" s="27"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="23" t="s">
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="11"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="M32" s="23"/>
-      <c r="N32" s="23"/>
-      <c r="O32" s="23"/>
-      <c r="P32" s="23"/>
+      <c r="M32" s="27"/>
+      <c r="N32" s="27"/>
+      <c r="O32" s="27"/>
+      <c r="P32" s="27"/>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="16" t="s">
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="12" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="8" t="s">
+      <c r="C34" s="7"/>
+      <c r="D34" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="16"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="12"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="8" t="s">
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="16"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="12"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="8" t="s">
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="16"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="12"/>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="16"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="12"/>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="16"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="12"/>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="18" t="s">
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="6" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="14"/>
-      <c r="D40" s="8" t="s">
+      <c r="C40" s="7"/>
+      <c r="D40" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="18"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="6"/>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="8" t="s">
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="18"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="6"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="8" t="s">
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="18"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="6"/>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="18"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="6"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="18"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="79">
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="D3:K3"/>
-    <mergeCell ref="D4:K4"/>
-    <mergeCell ref="B3:C6"/>
-    <mergeCell ref="B7:C9"/>
+    <mergeCell ref="J30:K32"/>
+    <mergeCell ref="J14:P14"/>
+    <mergeCell ref="L28:P28"/>
+    <mergeCell ref="L29:P29"/>
+    <mergeCell ref="L30:P30"/>
+    <mergeCell ref="L31:P31"/>
+    <mergeCell ref="L32:P32"/>
+    <mergeCell ref="J27:K29"/>
+    <mergeCell ref="L22:P22"/>
+    <mergeCell ref="L23:P23"/>
+    <mergeCell ref="L24:P24"/>
+    <mergeCell ref="L25:P25"/>
+    <mergeCell ref="L26:P26"/>
+    <mergeCell ref="L27:P27"/>
+    <mergeCell ref="L16:P16"/>
+    <mergeCell ref="L17:P17"/>
+    <mergeCell ref="L18:P18"/>
+    <mergeCell ref="L19:P19"/>
+    <mergeCell ref="L20:P20"/>
+    <mergeCell ref="L21:P21"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="O3:Q3"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="L15:P15"/>
+    <mergeCell ref="J17:K20"/>
+    <mergeCell ref="J24:K26"/>
+    <mergeCell ref="J21:K23"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="B19:G20"/>
+    <mergeCell ref="H15:H20"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="B25:G26"/>
+    <mergeCell ref="J15:K16"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:C18"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="B22:C24"/>
+    <mergeCell ref="H21:H26"/>
+    <mergeCell ref="B31:G32"/>
+    <mergeCell ref="H27:H32"/>
+    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B37:G38"/>
+    <mergeCell ref="H33:H38"/>
+    <mergeCell ref="B34:C36"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="D36:G36"/>
+    <mergeCell ref="B28:C30"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="B27:G27"/>
     <mergeCell ref="B10:C12"/>
     <mergeCell ref="D5:K5"/>
     <mergeCell ref="D6:K6"/>
@@ -1853,64 +1906,11 @@
     <mergeCell ref="D11:K11"/>
     <mergeCell ref="D12:K12"/>
     <mergeCell ref="B43:G44"/>
-    <mergeCell ref="B31:G32"/>
-    <mergeCell ref="H27:H32"/>
-    <mergeCell ref="B33:G33"/>
-    <mergeCell ref="B37:G38"/>
-    <mergeCell ref="H33:H38"/>
-    <mergeCell ref="B34:C36"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="D35:G35"/>
-    <mergeCell ref="D36:G36"/>
-    <mergeCell ref="B28:C30"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="B16:C18"/>
-    <mergeCell ref="D16:G16"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="B22:C24"/>
-    <mergeCell ref="H21:H26"/>
-    <mergeCell ref="J17:K20"/>
-    <mergeCell ref="J24:K26"/>
-    <mergeCell ref="J21:K23"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="B19:G20"/>
-    <mergeCell ref="H15:H20"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="B25:G26"/>
-    <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="O3:Q3"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="L15:P15"/>
-    <mergeCell ref="L17:P17"/>
-    <mergeCell ref="L18:P18"/>
-    <mergeCell ref="L19:P19"/>
-    <mergeCell ref="L20:P20"/>
-    <mergeCell ref="L21:P21"/>
-    <mergeCell ref="J15:K16"/>
-    <mergeCell ref="J30:K32"/>
-    <mergeCell ref="J14:P14"/>
-    <mergeCell ref="L28:P28"/>
-    <mergeCell ref="L29:P29"/>
-    <mergeCell ref="L30:P30"/>
-    <mergeCell ref="L31:P31"/>
-    <mergeCell ref="L32:P32"/>
-    <mergeCell ref="J27:K29"/>
-    <mergeCell ref="L22:P22"/>
-    <mergeCell ref="L23:P23"/>
-    <mergeCell ref="L24:P24"/>
-    <mergeCell ref="L25:P25"/>
-    <mergeCell ref="L26:P26"/>
-    <mergeCell ref="L27:P27"/>
-    <mergeCell ref="L16:P16"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="D3:K3"/>
+    <mergeCell ref="D4:K4"/>
+    <mergeCell ref="B3:C6"/>
+    <mergeCell ref="B7:C9"/>
   </mergeCells>
   <conditionalFormatting sqref="O2:Q5">
     <cfRule type="colorScale" priority="1">

</xml_diff>